<commit_message>
Update NFC_Reader.xlsx ODK form
Replace the NFC_Reader.xlsx ODK form with an updated binary version. The diff is binary so exact field-level changes are not shown here; this commit updates the form workbook contents and metadata.
</commit_message>
<xml_diff>
--- a/odk_form/NFC_Reader.xlsx
+++ b/odk_form/NFC_Reader.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/icrucrob/Desktop/odk-nfc-connector_V1/odk_form/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/icrucrob/Documents/GitHub/tagbridge_nfc/odk_form/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DC15DD76-2303-DA4F-8525-926E81B68E96}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E45F52C5-42F8-414A-9FA6-8AF209A200E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="1000" windowWidth="34560" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -3204,13 +3204,13 @@
     <t>body::intent</t>
   </si>
   <si>
-    <t>uk.ac.lshtm.odknfcconnector.SCAN_NFC(value_field='tag_id_hex')</t>
-  </si>
-  <si>
-    <t>uk.ac.lshtm.odknfcconnector.SCAN_NFC(value_field='tag_id_hex', return_fields='tag_id_hex,tag_id_dec,tech_list', format='json')</t>
-  </si>
-  <si>
-    <t>uk.ac.lshtm.odknfcconnector.SCAN_NFC</t>
+    <t>ex:uk.ac.lshtm.tagbridge.SCAN_NFC(value_field='tag_id_hex', return_fields='tag_id_hex,tag_id_dec,tech_list', format='json')</t>
+  </si>
+  <si>
+    <t>ex:uk.ac.lshtm.tagbridge.SCAN_NFC(value_field='tag_id_hex')</t>
+  </si>
+  <si>
+    <t>uk.ac.lshtm.tagbridge.SCAN_NFC</t>
   </si>
 </sst>
 </file>
@@ -4494,7 +4494,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="262">
+  <cellXfs count="259">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -4964,6 +4964,7 @@
     <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -4995,19 +4996,11 @@
     <xf numFmtId="0" fontId="5" fillId="7" borderId="61" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="38">
+  <dxfs count="33">
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -5103,51 +5096,6 @@
         <patternFill patternType="solid">
           <fgColor rgb="FF4A86E8"/>
           <bgColor rgb="FF4A86E8"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFB7E1CD"/>
-          <bgColor rgb="FFB7E1CD"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFFFFFFF"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF4A86E8"/>
-          <bgColor rgb="FF4A86E8"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFB7E1CD"/>
-          <bgColor rgb="FFB7E1CD"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFFFFFFF"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF4A86E8"/>
-          <bgColor rgb="FF4A86E8"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFF3F3F3"/>
         </patternFill>
       </fill>
     </dxf>
@@ -5325,37 +5273,37 @@
   </dxfs>
   <tableStyles count="7">
     <tableStyle name="survey-style" pivot="0" count="2" xr9:uid="{00000000-0011-0000-FFFF-FFFF00000000}">
-      <tableStyleElement type="firstRowStripe" dxfId="37"/>
-      <tableStyleElement type="secondRowStripe" dxfId="36"/>
-    </tableStyle>
-    <tableStyle name="choices-style" pivot="0" count="2" xr9:uid="{00000000-0011-0000-FFFF-FFFF01000000}">
-      <tableStyleElement type="firstRowStripe" dxfId="35"/>
-      <tableStyleElement type="secondRowStripe" dxfId="34"/>
-    </tableStyle>
-    <tableStyle name="🔀 Relevance-style" pivot="0" count="3" xr9:uid="{00000000-0011-0000-FFFF-FFFF02000000}">
-      <tableStyleElement type="headerRow" dxfId="33"/>
       <tableStyleElement type="firstRowStripe" dxfId="32"/>
       <tableStyleElement type="secondRowStripe" dxfId="31"/>
     </tableStyle>
+    <tableStyle name="choices-style" pivot="0" count="2" xr9:uid="{00000000-0011-0000-FFFF-FFFF01000000}">
+      <tableStyleElement type="firstRowStripe" dxfId="30"/>
+      <tableStyleElement type="secondRowStripe" dxfId="29"/>
+    </tableStyle>
+    <tableStyle name="🔀 Relevance-style" pivot="0" count="3" xr9:uid="{00000000-0011-0000-FFFF-FFFF02000000}">
+      <tableStyleElement type="headerRow" dxfId="28"/>
+      <tableStyleElement type="firstRowStripe" dxfId="27"/>
+      <tableStyleElement type="secondRowStripe" dxfId="26"/>
+    </tableStyle>
     <tableStyle name="🔒 Constraints-style" pivot="0" count="3" xr9:uid="{00000000-0011-0000-FFFF-FFFF03000000}">
-      <tableStyleElement type="headerRow" dxfId="30"/>
-      <tableStyleElement type="firstRowStripe" dxfId="29"/>
-      <tableStyleElement type="secondRowStripe" dxfId="28"/>
+      <tableStyleElement type="headerRow" dxfId="25"/>
+      <tableStyleElement type="firstRowStripe" dxfId="24"/>
+      <tableStyleElement type="secondRowStripe" dxfId="23"/>
     </tableStyle>
     <tableStyle name="✅ Additional columns-style" pivot="0" count="3" xr9:uid="{00000000-0011-0000-FFFF-FFFF04000000}">
-      <tableStyleElement type="headerRow" dxfId="27"/>
-      <tableStyleElement type="firstRowStripe" dxfId="26"/>
-      <tableStyleElement type="secondRowStripe" dxfId="25"/>
+      <tableStyleElement type="headerRow" dxfId="22"/>
+      <tableStyleElement type="firstRowStripe" dxfId="21"/>
+      <tableStyleElement type="secondRowStripe" dxfId="20"/>
     </tableStyle>
     <tableStyle name="✅ Additional columns-style 2" pivot="0" count="3" xr9:uid="{00000000-0011-0000-FFFF-FFFF05000000}">
-      <tableStyleElement type="headerRow" dxfId="24"/>
-      <tableStyleElement type="firstRowStripe" dxfId="23"/>
-      <tableStyleElement type="secondRowStripe" dxfId="22"/>
+      <tableStyleElement type="headerRow" dxfId="19"/>
+      <tableStyleElement type="firstRowStripe" dxfId="18"/>
+      <tableStyleElement type="secondRowStripe" dxfId="17"/>
     </tableStyle>
     <tableStyle name="✅ Additional columns-style 3" pivot="0" count="3" xr9:uid="{00000000-0011-0000-FFFF-FFFF06000000}">
-      <tableStyleElement type="headerRow" dxfId="21"/>
-      <tableStyleElement type="firstRowStripe" dxfId="20"/>
-      <tableStyleElement type="secondRowStripe" dxfId="19"/>
+      <tableStyleElement type="headerRow" dxfId="16"/>
+      <tableStyleElement type="firstRowStripe" dxfId="15"/>
+      <tableStyleElement type="secondRowStripe" dxfId="14"/>
     </tableStyle>
   </tableStyles>
   <colors>
@@ -5809,7 +5757,7 @@
       <c r="E2" s="237"/>
       <c r="F2" s="237"/>
       <c r="G2" s="232" t="s">
-        <v>620</v>
+        <v>621</v>
       </c>
       <c r="H2" s="237"/>
       <c r="I2" s="237"/>
@@ -5840,7 +5788,7 @@
       <c r="E3" s="237"/>
       <c r="F3" s="237"/>
       <c r="G3" s="232" t="s">
-        <v>621</v>
+        <v>620</v>
       </c>
       <c r="H3" s="237"/>
       <c r="I3" s="237"/>
@@ -5855,43 +5803,43 @@
       <c r="R3" s="237"/>
       <c r="S3" s="237"/>
     </row>
-    <row r="4" spans="1:24" s="261" customFormat="1" ht="56">
-      <c r="A4" s="259" t="s">
+    <row r="4" spans="1:24" s="239" customFormat="1" ht="56">
+      <c r="A4" s="2" t="s">
         <v>94</v>
       </c>
-      <c r="B4" s="258" t="s">
+      <c r="B4" s="3" t="s">
         <v>608</v>
       </c>
-      <c r="C4" s="259" t="s">
+      <c r="C4" s="2" t="s">
         <v>609</v>
       </c>
-      <c r="D4" s="259" t="s">
+      <c r="D4" s="2" t="s">
         <v>610</v>
       </c>
-      <c r="E4" s="259"/>
-      <c r="F4" s="259"/>
-      <c r="G4" s="261" t="s">
+      <c r="E4" s="2"/>
+      <c r="F4" s="2"/>
+      <c r="G4" s="239" t="s">
         <v>246</v>
       </c>
-      <c r="H4" s="259"/>
-      <c r="I4" s="259"/>
-      <c r="J4" s="259"/>
-      <c r="K4" s="259"/>
-      <c r="L4" s="259"/>
-      <c r="M4" s="259"/>
-      <c r="N4" s="259"/>
-      <c r="O4" s="259"/>
-      <c r="P4" s="259"/>
-      <c r="Q4" s="259"/>
-      <c r="R4" s="259"/>
-      <c r="S4" s="259"/>
+      <c r="H4" s="2"/>
+      <c r="I4" s="2"/>
+      <c r="J4" s="2"/>
+      <c r="K4" s="2"/>
+      <c r="L4" s="2"/>
+      <c r="M4" s="2"/>
+      <c r="N4" s="2"/>
+      <c r="O4" s="2"/>
+      <c r="P4" s="2"/>
+      <c r="Q4" s="2"/>
+      <c r="R4" s="2"/>
+      <c r="S4" s="2"/>
       <c r="T4" s="232" t="s">
         <v>622</v>
       </c>
-      <c r="U4" s="260"/>
-      <c r="V4" s="260"/>
-      <c r="W4" s="260"/>
-      <c r="X4" s="260"/>
+      <c r="U4" s="4"/>
+      <c r="V4" s="4"/>
+      <c r="W4" s="4"/>
+      <c r="X4" s="4"/>
     </row>
     <row r="5" spans="1:24" ht="15">
       <c r="A5" s="2" t="s">
@@ -18424,30 +18372,30 @@
   <sheetData>
     <row r="1" spans="1:12" ht="39" customHeight="1" thickBot="1">
       <c r="A1" s="98"/>
-      <c r="B1" s="253" t="s">
+      <c r="B1" s="254" t="s">
         <v>324</v>
       </c>
-      <c r="C1" s="246"/>
-      <c r="D1" s="246"/>
-      <c r="E1" s="246"/>
-      <c r="F1" s="246"/>
-      <c r="G1" s="246"/>
-      <c r="H1" s="246"/>
-      <c r="I1" s="246"/>
+      <c r="C1" s="247"/>
+      <c r="D1" s="247"/>
+      <c r="E1" s="247"/>
+      <c r="F1" s="247"/>
+      <c r="G1" s="247"/>
+      <c r="H1" s="247"/>
+      <c r="I1" s="247"/>
       <c r="J1" s="117"/>
       <c r="K1" s="37"/>
       <c r="L1" s="11"/>
     </row>
     <row r="2" spans="1:12" ht="14" thickBot="1">
       <c r="A2" s="37"/>
-      <c r="B2" s="254"/>
-      <c r="C2" s="255"/>
-      <c r="D2" s="255"/>
-      <c r="E2" s="255"/>
-      <c r="F2" s="255"/>
-      <c r="G2" s="255"/>
-      <c r="H2" s="255"/>
-      <c r="I2" s="255"/>
+      <c r="B2" s="255"/>
+      <c r="C2" s="256"/>
+      <c r="D2" s="256"/>
+      <c r="E2" s="256"/>
+      <c r="F2" s="256"/>
+      <c r="G2" s="256"/>
+      <c r="H2" s="256"/>
+      <c r="I2" s="256"/>
       <c r="J2" s="37"/>
       <c r="K2" s="37"/>
       <c r="L2" s="11"/>
@@ -30211,14 +30159,14 @@
   <sheetData>
     <row r="1" spans="1:8" ht="39" customHeight="1" thickBot="1">
       <c r="A1" s="98"/>
-      <c r="B1" s="253" t="s">
+      <c r="B1" s="254" t="s">
         <v>350</v>
       </c>
-      <c r="C1" s="246"/>
-      <c r="D1" s="246"/>
-      <c r="E1" s="246"/>
-      <c r="F1" s="246"/>
-      <c r="G1" s="246"/>
+      <c r="C1" s="247"/>
+      <c r="D1" s="247"/>
+      <c r="E1" s="247"/>
+      <c r="F1" s="247"/>
+      <c r="G1" s="247"/>
       <c r="H1" s="37"/>
     </row>
     <row r="2" spans="1:8" ht="14" thickBot="1">
@@ -30469,13 +30417,13 @@
     </row>
     <row r="22" spans="1:8" ht="14">
       <c r="A22" s="165"/>
-      <c r="B22" s="256" t="s">
+      <c r="B22" s="257" t="s">
         <v>370</v>
       </c>
-      <c r="C22" s="255"/>
-      <c r="D22" s="255"/>
-      <c r="E22" s="255"/>
-      <c r="F22" s="255"/>
+      <c r="C22" s="256"/>
+      <c r="D22" s="256"/>
+      <c r="E22" s="256"/>
+      <c r="F22" s="256"/>
       <c r="G22" s="169" t="s">
         <v>371</v>
       </c>
@@ -30483,13 +30431,13 @@
     </row>
     <row r="23" spans="1:8" ht="28">
       <c r="A23" s="165"/>
-      <c r="B23" s="257" t="s">
+      <c r="B23" s="258" t="s">
         <v>372</v>
       </c>
-      <c r="C23" s="255"/>
-      <c r="D23" s="255"/>
-      <c r="E23" s="255"/>
-      <c r="F23" s="255"/>
+      <c r="C23" s="256"/>
+      <c r="D23" s="256"/>
+      <c r="E23" s="256"/>
+      <c r="F23" s="256"/>
       <c r="G23" s="170" t="s">
         <v>373</v>
       </c>
@@ -30497,13 +30445,13 @@
     </row>
     <row r="24" spans="1:8" ht="28">
       <c r="A24" s="165"/>
-      <c r="B24" s="256" t="s">
+      <c r="B24" s="257" t="s">
         <v>374</v>
       </c>
-      <c r="C24" s="255"/>
-      <c r="D24" s="255"/>
-      <c r="E24" s="255"/>
-      <c r="F24" s="255"/>
+      <c r="C24" s="256"/>
+      <c r="D24" s="256"/>
+      <c r="E24" s="256"/>
+      <c r="F24" s="256"/>
       <c r="G24" s="169" t="s">
         <v>375</v>
       </c>
@@ -30511,13 +30459,13 @@
     </row>
     <row r="25" spans="1:8" ht="28">
       <c r="A25" s="171"/>
-      <c r="B25" s="257" t="s">
+      <c r="B25" s="258" t="s">
         <v>376</v>
       </c>
-      <c r="C25" s="255"/>
-      <c r="D25" s="255"/>
-      <c r="E25" s="255"/>
-      <c r="F25" s="255"/>
+      <c r="C25" s="256"/>
+      <c r="D25" s="256"/>
+      <c r="E25" s="256"/>
+      <c r="F25" s="256"/>
       <c r="G25" s="170" t="s">
         <v>377</v>
       </c>
@@ -30525,13 +30473,13 @@
     </row>
     <row r="26" spans="1:8" ht="14">
       <c r="A26" s="165"/>
-      <c r="B26" s="256" t="s">
+      <c r="B26" s="257" t="s">
         <v>378</v>
       </c>
-      <c r="C26" s="255"/>
-      <c r="D26" s="255"/>
-      <c r="E26" s="255"/>
-      <c r="F26" s="255"/>
+      <c r="C26" s="256"/>
+      <c r="D26" s="256"/>
+      <c r="E26" s="256"/>
+      <c r="F26" s="256"/>
       <c r="G26" s="169" t="s">
         <v>379</v>
       </c>
@@ -30539,13 +30487,13 @@
     </row>
     <row r="27" spans="1:8" ht="42">
       <c r="A27" s="165"/>
-      <c r="B27" s="257" t="s">
+      <c r="B27" s="258" t="s">
         <v>380</v>
       </c>
-      <c r="C27" s="255"/>
-      <c r="D27" s="255"/>
-      <c r="E27" s="255"/>
-      <c r="F27" s="255"/>
+      <c r="C27" s="256"/>
+      <c r="D27" s="256"/>
+      <c r="E27" s="256"/>
+      <c r="F27" s="256"/>
       <c r="G27" s="170" t="s">
         <v>381</v>
       </c>
@@ -39910,14 +39858,14 @@
   <sheetData>
     <row r="1" spans="1:8" ht="33" customHeight="1">
       <c r="A1" s="178"/>
-      <c r="B1" s="253" t="s">
+      <c r="B1" s="254" t="s">
         <v>390</v>
       </c>
-      <c r="C1" s="246"/>
-      <c r="D1" s="246"/>
-      <c r="E1" s="246"/>
-      <c r="F1" s="246"/>
-      <c r="G1" s="246"/>
+      <c r="C1" s="247"/>
+      <c r="D1" s="247"/>
+      <c r="E1" s="247"/>
+      <c r="F1" s="247"/>
+      <c r="G1" s="247"/>
       <c r="H1" s="28"/>
     </row>
     <row r="2" spans="1:8" ht="13">
@@ -46054,7 +46002,7 @@
       <c r="B2" s="11"/>
       <c r="C2" s="11" t="str">
         <f ca="1">TEXT(NOW(), "yyyymmddhhmmss")</f>
-        <v>20260511123849</v>
+        <v>20260511131644</v>
       </c>
       <c r="D2" s="11"/>
       <c r="E2" s="11"/>
@@ -58056,11 +58004,11 @@
   <sheetData>
     <row r="1" spans="1:10" ht="27.75" customHeight="1">
       <c r="A1" s="12"/>
-      <c r="B1" s="239"/>
-      <c r="C1" s="241" t="s">
+      <c r="B1" s="240"/>
+      <c r="C1" s="242" t="s">
         <v>26</v>
       </c>
-      <c r="D1" s="242"/>
+      <c r="D1" s="243"/>
       <c r="E1" s="12"/>
       <c r="F1" s="12"/>
       <c r="G1" s="13"/>
@@ -58074,9 +58022,9 @@
     </row>
     <row r="2" spans="1:10" ht="21.75" customHeight="1">
       <c r="A2" s="12"/>
-      <c r="B2" s="240"/>
-      <c r="C2" s="243"/>
-      <c r="D2" s="244"/>
+      <c r="B2" s="241"/>
+      <c r="C2" s="244"/>
+      <c r="D2" s="245"/>
       <c r="E2" s="16"/>
       <c r="F2" s="16"/>
       <c r="G2" s="17"/>
@@ -58648,22 +58596,22 @@
   <sheetData>
     <row r="1" spans="1:7" ht="39" customHeight="1">
       <c r="A1" s="36"/>
-      <c r="B1" s="245" t="s">
+      <c r="B1" s="246" t="s">
         <v>60</v>
       </c>
-      <c r="C1" s="246"/>
-      <c r="D1" s="246"/>
-      <c r="E1" s="246"/>
-      <c r="F1" s="246"/>
+      <c r="C1" s="247"/>
+      <c r="D1" s="247"/>
+      <c r="E1" s="247"/>
+      <c r="F1" s="247"/>
       <c r="G1" s="37"/>
     </row>
     <row r="2" spans="1:7" ht="13">
       <c r="A2" s="37"/>
-      <c r="B2" s="247"/>
-      <c r="C2" s="248"/>
-      <c r="D2" s="248"/>
-      <c r="E2" s="248"/>
-      <c r="F2" s="249"/>
+      <c r="B2" s="248"/>
+      <c r="C2" s="249"/>
+      <c r="D2" s="249"/>
+      <c r="E2" s="249"/>
+      <c r="F2" s="250"/>
       <c r="G2" s="37"/>
     </row>
     <row r="3" spans="1:7" ht="13">
@@ -59461,22 +59409,22 @@
   <sheetData>
     <row r="1" spans="1:7" ht="41.25" customHeight="1">
       <c r="A1" s="74"/>
-      <c r="B1" s="245" t="s">
+      <c r="B1" s="246" t="s">
         <v>155</v>
       </c>
-      <c r="C1" s="246"/>
-      <c r="D1" s="246"/>
-      <c r="E1" s="246"/>
-      <c r="F1" s="246"/>
+      <c r="C1" s="247"/>
+      <c r="D1" s="247"/>
+      <c r="E1" s="247"/>
+      <c r="F1" s="247"/>
       <c r="G1" s="75"/>
     </row>
     <row r="2" spans="1:7" ht="13">
       <c r="A2" s="75"/>
-      <c r="B2" s="250"/>
-      <c r="C2" s="251"/>
-      <c r="D2" s="251"/>
-      <c r="E2" s="251"/>
-      <c r="F2" s="252"/>
+      <c r="B2" s="251"/>
+      <c r="C2" s="252"/>
+      <c r="D2" s="252"/>
+      <c r="E2" s="252"/>
+      <c r="F2" s="253"/>
       <c r="G2" s="75"/>
     </row>
     <row r="3" spans="1:7" ht="13">
@@ -60445,10 +60393,10 @@
   <sheetData>
     <row r="1" spans="1:4" ht="39.75" customHeight="1" thickBot="1">
       <c r="A1" s="98"/>
-      <c r="B1" s="245" t="s">
+      <c r="B1" s="246" t="s">
         <v>265</v>
       </c>
-      <c r="C1" s="246"/>
+      <c r="C1" s="247"/>
       <c r="D1" s="99"/>
     </row>
     <row r="2" spans="1:4" ht="14" thickBot="1">
@@ -60640,10 +60588,10 @@
   <sheetData>
     <row r="1" spans="1:4" ht="38.25" customHeight="1" thickBot="1">
       <c r="A1" s="74"/>
-      <c r="B1" s="245" t="s">
+      <c r="B1" s="246" t="s">
         <v>291</v>
       </c>
-      <c r="C1" s="246"/>
+      <c r="C1" s="247"/>
       <c r="D1" s="75"/>
     </row>
     <row r="2" spans="1:4" ht="14" thickBot="1">

</xml_diff>